<commit_message>
Adding Reports and other
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/TaskCreationTestData.xlsx
+++ b/src/test/resources/testData/TaskCreationTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vishal\Desktop\SeleniumAutomation\eclipse-workspace\AdvanceFrameWorkDesign\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E203D44F-3186-43D8-9DBC-3A7F123BAC5B}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB197A4-3E8D-447C-9D4B-0B0CF59116CD}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{5F7D3B99-D034-441B-B1F7-06ED4F3CD305}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="67">
   <si>
     <t>Sr No</t>
   </si>
@@ -184,15 +184,9 @@
     <t>Vaibhav</t>
   </si>
   <si>
-    <t>Sayali</t>
-  </si>
-  <si>
     <t>Shaha</t>
   </si>
   <si>
-    <t>Mehta</t>
-  </si>
-  <si>
     <t>Married</t>
   </si>
   <si>
@@ -239,6 +233,9 @@
   </si>
   <si>
     <t>Dance,Reading</t>
+  </si>
+  <si>
+    <t>Aaryan</t>
   </si>
 </sst>
 </file>
@@ -858,16 +855,16 @@
         <v>47</v>
       </c>
       <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" t="s">
         <v>50</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>52</v>
       </c>
-      <c r="E2" t="s">
-        <v>54</v>
-      </c>
       <c r="F2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -882,19 +879,19 @@
         <v>6572537422</v>
       </c>
       <c r="K2" t="s">
+        <v>54</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="M2" t="s">
         <v>56</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" t="s">
         <v>57</v>
       </c>
-      <c r="M2" t="s">
-        <v>58</v>
-      </c>
-      <c r="N2" t="s">
-        <v>59</v>
-      </c>
       <c r="O2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -905,16 +902,16 @@
         <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" t="s">
         <v>53</v>
-      </c>
-      <c r="E3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F3" t="s">
-        <v>55</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -929,19 +926,19 @@
         <v>6572537429</v>
       </c>
       <c r="K3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="M3" t="s">
+        <v>62</v>
+      </c>
+      <c r="N3" t="s">
         <v>60</v>
       </c>
-      <c r="L3" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M3" t="s">
-        <v>64</v>
-      </c>
-      <c r="N3" t="s">
-        <v>62</v>
-      </c>
       <c r="O3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -949,19 +946,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" t="s">
         <v>49</v>
       </c>
-      <c r="C4" t="s">
-        <v>51</v>
-      </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -976,19 +973,19 @@
         <v>6572537428</v>
       </c>
       <c r="K4" t="s">
+        <v>59</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="M4" t="s">
+        <v>63</v>
+      </c>
+      <c r="N4" t="s">
         <v>61</v>
       </c>
-      <c r="L4" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M4" t="s">
-        <v>65</v>
-      </c>
-      <c r="N4" t="s">
-        <v>63</v>
-      </c>
       <c r="O4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>